<commit_message>
refactor: rename example outcomes to match brcharts publication
Rename the generic outcome labels to the names used in the earlier
brcharts publication (corr dataset spelling):

  Benefit 1 -> Primary Efficacy
  Benefit 2 -> Secondary Efficacy
  Benefit 3 -> Quality of Life
  Risk 1    -> Recurring AE
  Risk 2    -> Rare SAE
  Risk 3    -> Liver Toxicity

- Update the Outcome column in data-raw/Manuscript_Generic_Example.xlsx
  and regenerate effects_table, mcda_data, corr, clinical_scales and
  weights (values unchanged, names only)
- Fix effects_table row 12 (Drug B, Toxicity), which was mislabelled
  as Risk 2 instead of Risk 3
- Update R source, roxygen/man pages, tests, vignettes and README
- Replace stale head(mcda_data) example output in the roxygen comments

Refs #73

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/Manuscript_Generic_Example.xlsx
+++ b/data-raw/Manuscript_Generic_Example.xlsx
@@ -635,22 +635,22 @@
     <t>Drug D</t>
   </si>
   <si>
-    <t>Benefit 1</t>
-  </si>
-  <si>
-    <t>Benefit 2</t>
-  </si>
-  <si>
-    <t>Benefit 3</t>
-  </si>
-  <si>
-    <t>Risk 1</t>
-  </si>
-  <si>
-    <t>Risk 2</t>
-  </si>
-  <si>
-    <t>Risk 3</t>
+    <t>Primary Efficacy</t>
+  </si>
+  <si>
+    <t>Secondary Efficacy</t>
+  </si>
+  <si>
+    <t>Quality of Life</t>
+  </si>
+  <si>
+    <t>Recurring AE</t>
+  </si>
+  <si>
+    <t>Rare SAE</t>
+  </si>
+  <si>
+    <t>Liver Toxicity</t>
   </si>
 </sst>
 </file>
@@ -2253,7 +2253,7 @@
         <v>175</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D13" s="30" t="s">
         <v>178</v>

</xml_diff>